<commit_message>
feat: migrate web and Android interfaces to BioFlow
</commit_message>
<xml_diff>
--- a/documentation/BiovitAI-Documentation-v2.1/project-management/BiovitAI_v2_1_Development_Tracker.xlsx
+++ b/documentation/BiovitAI-Documentation-v2.1/project-management/BiovitAI_v2_1_Development_Tracker.xlsx
@@ -1,14 +1,5 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb61ede562ffb43de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R45668e30ceb14a4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phases" sheetId="3" r:id="R7cba5b612914497d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rec68ed25c01249c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="5" r:id="R696fc783942d4219"/>
-  </x:sheets>
-</x:workbook>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="UTF-8"?><x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"><x:sheets><x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb61ede562ffb43de"/><x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R45668e30ceb14a4d"/><x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phases" sheetId="3" r:id="R7cba5b612914497d"/><x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rec68ed25c01249c4"/><x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="5" r:id="R696fc783942d4219"/><sheet name="BioFlow" sheetId="6" r:id="rIdBioFlow"/></x:sheets></x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -20,7 +11,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -61,8 +52,40 @@
       <x:color rgb="FF13243A"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="17"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="17"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -94,15 +117,33 @@
         <x:fgColor rgb="FFDBEAF0"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF087F82"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="3">
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="51">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -171,6 +212,23 @@
     <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="0"/>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -5630,4 +5688,242 @@
     <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a2b14bf2c7242c1"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="38" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="66" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="43" t="str">
+        <x:v>BioFlow UI migration</x:v>
+      </x:c>
+      <x:c r="B1" s="41"/>
+      <x:c r="C1" s="41"/>
+      <x:c r="D1" s="41"/>
+      <x:c r="E1" s="41"/>
+      <x:c r="F1" s="41"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="41" t="str">
+        <x:v>Engineering progress. The original 51 task records and formal review statuses are retained.</x:v>
+      </x:c>
+      <x:c r="B2" s="41"/>
+      <x:c r="C2" s="41"/>
+      <x:c r="D2" s="41"/>
+      <x:c r="E2" s="41"/>
+      <x:c r="F2" s="41"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="41"/>
+      <x:c r="B3" s="41"/>
+      <x:c r="C3" s="41"/>
+      <x:c r="D3" s="41"/>
+      <x:c r="E3" s="41"/>
+      <x:c r="F3" s="41"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="47" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B4" s="47" t="str">
+        <x:v>Workstream</x:v>
+      </x:c>
+      <x:c r="C4" s="47" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="D4" s="47" t="str">
+        <x:v>Related Tasks</x:v>
+      </x:c>
+      <x:c r="E4" s="47" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="F4" s="47" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="70" customHeight="1">
+      <x:c r="A5" s="49" t="str">
+        <x:v>BF-001</x:v>
+      </x:c>
+      <x:c r="B5" s="49" t="str">
+        <x:v>Inventory and design system</x:v>
+      </x:c>
+      <x:c r="C5" s="49" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D5" s="49" t="str">
+        <x:v>BV-001; BV-012</x:v>
+      </x:c>
+      <x:c r="E5" s="49" t="str">
+        <x:v>documentation/design-system/VALIDATION-REPORT.md</x:v>
+      </x:c>
+      <x:c r="F5" s="49" t="str">
+        <x:v>Inventory covers 111 discovered surfaces; shared tokens, licensed local fonts, primitives and drift guards implemented. Validation is recorded separately.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="70" customHeight="1">
+      <x:c r="A6" s="49" t="str">
+        <x:v>BF-002</x:v>
+      </x:c>
+      <x:c r="B6" s="49" t="str">
+        <x:v>Web shell and dashboard</x:v>
+      </x:c>
+      <x:c r="C6" s="49" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D6" s="49" t="str">
+        <x:v>BV-012; BV-019; BV-020</x:v>
+      </x:c>
+      <x:c r="E6" s="49" t="str">
+        <x:v>documentation/design-system/VALIDATION-REPORT.md</x:v>
+      </x:c>
+      <x:c r="F6" s="49" t="str">
+        <x:v>Expanded web shell, actual evidence dashboard, neutral body, authorized search, filters and provenance implemented. Chromium and WebKit audits passed.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="70" customHeight="1">
+      <x:c r="A7" s="49" t="str">
+        <x:v>BF-003</x:v>
+      </x:c>
+      <x:c r="B7" s="49" t="str">
+        <x:v>Reports and health evidence</x:v>
+      </x:c>
+      <x:c r="C7" s="49" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D7" s="49" t="str">
+        <x:v>BV-014–BV-023</x:v>
+      </x:c>
+      <x:c r="E7" s="49" t="str">
+        <x:v>documentation/design-system/VALIDATION-REPORT.md</x:v>
+      </x:c>
+      <x:c r="F7" s="49" t="str">
+        <x:v>Real scanner/OCR production journey passed upload, identity, verify, append correction, compare and source. Rare UI branches remain explicit in coverage.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="70" customHeight="1">
+      <x:c r="A8" s="49" t="str">
+        <x:v>BF-004</x:v>
+      </x:c>
+      <x:c r="B8" s="49" t="str">
+        <x:v>Android migration</x:v>
+      </x:c>
+      <x:c r="C8" s="49" t="str">
+        <x:v>In Review</x:v>
+      </x:c>
+      <x:c r="D8" s="49" t="str">
+        <x:v>BV-012; BV-014–BV-028</x:v>
+      </x:c>
+      <x:c r="E8" s="49" t="str">
+        <x:v>documentation/design-system/VALIDATION-REPORT.md</x:v>
+      </x:c>
+      <x:c r="F8" s="49" t="str">
+        <x:v>APK/export, full emulator report/chat, comparison, caregiver revocation, focused routes and 150% text passed. TalkBack service smoke passed; manual/device acceptance remains pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="70" customHeight="1">
+      <x:c r="A9" s="49" t="str">
+        <x:v>BF-005</x:v>
+      </x:c>
+      <x:c r="B9" s="49" t="str">
+        <x:v>AI, profiles and supporting UI</x:v>
+      </x:c>
+      <x:c r="C9" s="49" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D9" s="49" t="str">
+        <x:v>BV-009; BV-024–BV-028</x:v>
+      </x:c>
+      <x:c r="E9" s="49" t="str">
+        <x:v>documentation/design-system/VALIDATION-REPORT.md</x:v>
+      </x:c>
+      <x:c r="F9" s="49" t="str">
+        <x:v>Auth/recovery, family/contact controls, consent/chat and honest unavailable/paused states migrated. Live AI presentation still requires configured provider.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="70" customHeight="1">
+      <x:c r="A10" s="49" t="str">
+        <x:v>BF-006</x:v>
+      </x:c>
+      <x:c r="B10" s="49" t="str">
+        <x:v>Regression and design QA</x:v>
+      </x:c>
+      <x:c r="C10" s="49" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="D10" s="49" t="str">
+        <x:v>BV-029–BV-031</x:v>
+      </x:c>
+      <x:c r="E10" s="49" t="str">
+        <x:v>documentation/design-system/VALIDATION-REPORT.md</x:v>
+      </x:c>
+      <x:c r="F10" s="49" t="str">
+        <x:v>51 core and 59 DB tests pass; production Chromium and WebKit gates pass. Firefox runtime, manual screen-reader/native RTL and physical-device validation remain pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="70" customHeight="1">
+      <x:c r="A11" s="49" t="str">
+        <x:v>BF-007</x:v>
+      </x:c>
+      <x:c r="B11" s="49" t="str">
+        <x:v>Coverage and governance</x:v>
+      </x:c>
+      <x:c r="C11" s="49" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D11" s="49" t="str">
+        <x:v>BV-001; BV-012; BV-031</x:v>
+      </x:c>
+      <x:c r="E11" s="49" t="str">
+        <x:v>documentation/design-system/VALIDATION-REPORT.md</x:v>
+      </x:c>
+      <x:c r="F11" s="49" t="str">
+        <x:v>All surfaces source-reviewed and accounted; coverage dimensions and limitations retained. Original 51 tasks, decisions, workbook sheets and formal review statuses preserved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="41"/>
+      <x:c r="B12" s="41"/>
+      <x:c r="C12" s="41"/>
+      <x:c r="D12" s="41"/>
+      <x:c r="E12" s="41"/>
+      <x:c r="F12" s="41"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="50" t="str">
+        <x:v>Source: Owner-approved BioFlow plan and recorded implementation evidence, 21 October 2026.</x:v>
+      </x:c>
+      <x:c r="B13" s="41"/>
+      <x:c r="C13" s="41"/>
+      <x:c r="D13" s="41"/>
+      <x:c r="E13" s="41"/>
+      <x:c r="F13" s="41"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="50" t="str">
+        <x:v>Checkpoint: https://github.com/FutureTechStudio/BioVitAI/commit/ced0d80bfe70d81258acadf63eca85b06fb2a9ba</x:v>
+      </x:c>
+      <x:c r="B14" s="41"/>
+      <x:c r="C14" s="41"/>
+      <x:c r="D14" s="41"/>
+      <x:c r="E14" s="41"/>
+      <x:c r="F14" s="41"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="C5:C11">
+      <x:formula1>"Backlog,Ready,In Progress,In Review,Done,Blocked"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: refine BioFlow profiles, floating assistant and tab layouts
</commit_message>
<xml_diff>
--- a/documentation/BiovitAI-Documentation-v2.1/project-management/BiovitAI_v2_1_Development_Tracker.xlsx
+++ b/documentation/BiovitAI-Documentation-v2.1/project-management/BiovitAI_v2_1_Development_Tracker.xlsx
@@ -5750,7 +5750,7 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="70" customHeight="1">
+    <x:row r="5" ht="82" customHeight="1">
       <x:c r="A5" s="49" t="str">
         <x:v>BF-001</x:v>
       </x:c>
@@ -5767,10 +5767,10 @@
         <x:v>documentation/design-system/VALIDATION-REPORT.md</x:v>
       </x:c>
       <x:c r="F5" s="49" t="str">
-        <x:v>Inventory covers 111 discovered surfaces; shared tokens, licensed local fonts, primitives and drift guards implemented. Validation is recorded separately.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="70" customHeight="1">
+        <x:v>Inventory covers 118 discovered surfaces; shared role-based tokens, licensed local fonts, primitives and drift guards implemented. Validation dimensions remain separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="82" customHeight="1">
       <x:c r="A6" s="49" t="str">
         <x:v>BF-002</x:v>
       </x:c>
@@ -5787,10 +5787,10 @@
         <x:v>documentation/design-system/VALIDATION-REPORT.md</x:v>
       </x:c>
       <x:c r="F6" s="49" t="str">
-        <x:v>Expanded web shell, actual evidence dashboard, neutral body, authorized search, filters and provenance implemented. Chromium and WebKit audits passed.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="70" customHeight="1">
+        <x:v>Avatar profile menu replaces in-page strip. Six distinct tab layouts use restrained green, blue, amber/coral and violet accents. Floating assistant replaces sidebar entry.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="82" customHeight="1">
       <x:c r="A7" s="49" t="str">
         <x:v>BF-003</x:v>
       </x:c>
@@ -5810,7 +5810,7 @@
         <x:v>Real scanner/OCR production journey passed upload, identity, verify, append correction, compare and source. Rare UI branches remain explicit in coverage.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="70" customHeight="1">
+    <x:row r="8" ht="82" customHeight="1">
       <x:c r="A8" s="49" t="str">
         <x:v>BF-004</x:v>
       </x:c>
@@ -5830,7 +5830,7 @@
         <x:v>APK/export, full emulator report/chat, comparison, caregiver revocation, focused routes and 150% text passed. TalkBack service smoke passed; manual/device acceptance remains pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="70" customHeight="1">
+    <x:row r="9" ht="82" customHeight="1">
       <x:c r="A9" s="49" t="str">
         <x:v>BF-005</x:v>
       </x:c>
@@ -5847,10 +5847,10 @@
         <x:v>documentation/design-system/VALIDATION-REPORT.md</x:v>
       </x:c>
       <x:c r="F9" s="49" t="str">
-        <x:v>Auth/recovery, family/contact controls, consent/chat and honest unavailable/paused states migrated. Live AI presentation still requires configured provider.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="70" customHeight="1">
+        <x:v>Session-scoped floating chat resumes current conversation; New chat, full-screen history, fresh sign-in and private profile resets covered. Email-less family/contact and consent flows retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="82" customHeight="1">
       <x:c r="A10" s="49" t="str">
         <x:v>BF-006</x:v>
       </x:c>
@@ -5867,10 +5867,10 @@
         <x:v>documentation/design-system/VALIDATION-REPORT.md</x:v>
       </x:c>
       <x:c r="F10" s="49" t="str">
-        <x:v>51 core and 59 DB tests pass; production Chromium and WebKit gates pass. Firefox runtime, manual screen-reader/native RTL and physical-device validation remain pending.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="70" customHeight="1">
+        <x:v>51 core tests and all five current production Chromium journeys pass; two current WebKit audits pass. Prior 59 DB regressions retained; Firefox, manual screen-reader and physical-device acceptance remain pending.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="82" customHeight="1">
       <x:c r="A11" s="49" t="str">
         <x:v>BF-007</x:v>
       </x:c>
@@ -5887,7 +5887,7 @@
         <x:v>documentation/design-system/VALIDATION-REPORT.md</x:v>
       </x:c>
       <x:c r="F11" s="49" t="str">
-        <x:v>All surfaces source-reviewed and accounted; coverage dimensions and limitations retained. Original 51 tasks, decisions, workbook sheets and formal review statuses preserved.</x:v>
+        <x:v>115 applicable surfaces source-reviewed out of 118 registered; coverage dimensions and limitations retained. Original 51 tasks, decisions, workbook sheets and formal review statuses preserved.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -5900,7 +5900,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="50" t="str">
-        <x:v>Source: Owner-approved BioFlow plan and recorded implementation evidence, 21 October 2026.</x:v>
+        <x:v>Source: Owner-approved BioFlow plan and recorded implementation evidence, 22 October 2026.</x:v>
       </x:c>
       <x:c r="B13" s="41"/>
       <x:c r="C13" s="41"/>

</xml_diff>

<commit_message>
feat: connect health story, context and change digest
</commit_message>
<xml_diff>
--- a/documentation/BiovitAI-Documentation-v2.1/project-management/BiovitAI_v2_1_Development_Tracker.xlsx
+++ b/documentation/BiovitAI-Documentation-v2.1/project-management/BiovitAI_v2_1_Development_Tracker.xlsx
@@ -1,5 +1,16 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="UTF-8"?><x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"><x:sheets><x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb61ede562ffb43de"/><x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R45668e30ceb14a4d"/><x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phases" sheetId="3" r:id="R7cba5b612914497d"/><x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rec68ed25c01249c4"/><x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="5" r:id="R696fc783942d4219"/><sheet name="BioFlow" sheetId="6" r:id="rIdBioFlow"/></x:sheets></x:workbook>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheets>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb61ede562ffb43de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" r:id="R45668e30ceb14a4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phases" sheetId="3" r:id="R7cba5b612914497d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rec68ed25c01249c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dependencies" sheetId="5" r:id="R696fc783942d4219"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BioFlow" sheetId="6" r:id="rIdBioFlow"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Journey" sheetId="7" r:id="rIdJourney"/>
+  </x:sheets>
+</x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11,7 +22,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="21">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -84,8 +95,40 @@
       <x:sz val="10"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="18"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="18"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="15">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -128,10 +171,38 @@
         <x:fgColor rgb="FF087F82"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF087F82"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF8F5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFCFEFE2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="3">
+  <x:borders count="4">
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
     <x:border>
       <x:left/>
       <x:right/>
@@ -143,7 +214,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="63">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -229,6 +300,26 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="13" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="10" borderId="3" xfId="0"/>
+    <x:xf numFmtId="0" fontId="15" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -5926,4 +6017,526 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="49" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="32" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="43" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="54" t="str">
+        <x:v>Connected health journey</x:v>
+      </x:c>
+      <x:c r="B1" s="52"/>
+      <x:c r="C1" s="52"/>
+      <x:c r="D1" s="52"/>
+      <x:c r="E1" s="52"/>
+      <x:c r="F1" s="52"/>
+      <x:c r="G1" s="52"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="52" t="str">
+        <x:v>Local engineering progress • 22 October 2026 • Original BV tasks and formal approvals unchanged</x:v>
+      </x:c>
+      <x:c r="B2" s="52"/>
+      <x:c r="C2" s="52"/>
+      <x:c r="D2" s="52"/>
+      <x:c r="E2" s="52"/>
+      <x:c r="F2" s="52"/>
+      <x:c r="G2" s="52"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="52"/>
+      <x:c r="B3" s="52"/>
+      <x:c r="C3" s="52"/>
+      <x:c r="D3" s="52"/>
+      <x:c r="E3" s="52"/>
+      <x:c r="F3" s="52"/>
+      <x:c r="G3" s="52"/>
+    </x:row>
+    <x:row r="4" ht="30" customHeight="1">
+      <x:c r="A4" s="57" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="B4" s="57" t="str">
+        <x:v>Workstream</x:v>
+      </x:c>
+      <x:c r="C4" s="57" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="D4" s="57" t="str">
+        <x:v>Dependencies</x:v>
+      </x:c>
+      <x:c r="E4" s="57" t="str">
+        <x:v>Related Tasks</x:v>
+      </x:c>
+      <x:c r="F4" s="57" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="G4" s="57" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="108" customHeight="1">
+      <x:c r="A5" s="60" t="str">
+        <x:v>CJ-001</x:v>
+      </x:c>
+      <x:c r="B5" s="60" t="str">
+        <x:v>Experience/domain contracts: record authority, date precision, source types, permission/consent matrix, route ownership and fact/claim language.</x:v>
+      </x:c>
+      <x:c r="C5" s="61" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D5" s="60" t="str">
+        <x:v>Current source baseline</x:v>
+      </x:c>
+      <x:c r="E5" s="60" t="str">
+        <x:v>BV-009–BV-013; BV-019–BV-028</x:v>
+      </x:c>
+      <x:c r="F5" s="60" t="str">
+        <x:v>docs/engineering/HEALTH-STORY-1.md</x:v>
+      </x:c>
+      <x:c r="G5" s="60" t="str">
+        <x:v>Health Story 1 local engineering complete: web/native journeys, permissions, encryption and restore verified. Clinical activation, manual accessibility, physical devices and participant signoff remain separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="108" customHeight="1">
+      <x:c r="A6" s="59" t="str">
+        <x:v>CJ-002</x:v>
+      </x:c>
+      <x:c r="B6" s="59" t="str">
+        <x:v>Typed conditions/medication/allergy/context assertions and documented instructions; confirmation/conflict workflow.</x:v>
+      </x:c>
+      <x:c r="C6" s="61" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D6" s="59" t="str">
+        <x:v>CJ-001</x:v>
+      </x:c>
+      <x:c r="E6" s="59" t="str">
+        <x:v>Health scope extension; BV-010</x:v>
+      </x:c>
+      <x:c r="F6" s="59" t="str">
+        <x:v>docs/engineering/HEALTH-STORY-1.md</x:v>
+      </x:c>
+      <x:c r="G6" s="59" t="str">
+        <x:v>Health Story 1 local engineering complete: web/native journeys, permissions, encryption and restore verified. Clinical activation, manual accessibility, physical devices and participant signoff remain separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="108" customHeight="1">
+      <x:c r="A7" s="60" t="str">
+        <x:v>CJ-003</x:v>
+      </x:c>
+      <x:c r="B7" s="60" t="str">
+        <x:v>Journey projection, existing-report backfill, timeline filters, source drilldown and undated lane.</x:v>
+      </x:c>
+      <x:c r="C7" s="61" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D7" s="60" t="str">
+        <x:v>CJ-001; CJ-002 for new context kinds</x:v>
+      </x:c>
+      <x:c r="E7" s="60" t="str">
+        <x:v>BV-010; BV-019–BV-023</x:v>
+      </x:c>
+      <x:c r="F7" s="60" t="str">
+        <x:v>docs/engineering/HEALTH-STORY-1.md</x:v>
+      </x:c>
+      <x:c r="G7" s="60" t="str">
+        <x:v>Health Story 1 local engineering complete: web/native journeys, permissions, encryption and restore verified. Clinical activation, manual accessibility, physical devices and participant signoff remain separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="108" customHeight="1">
+      <x:c r="A8" s="59" t="str">
+        <x:v>CJ-004</x:v>
+      </x:c>
+      <x:c r="B8" s="59" t="str">
+        <x:v>Change digest, actor review checkpoint, workflow/user priority queue and Dashboard simplification.</x:v>
+      </x:c>
+      <x:c r="C8" s="61" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="D8" s="59" t="str">
+        <x:v>CJ-003</x:v>
+      </x:c>
+      <x:c r="E8" s="59" t="str">
+        <x:v>BV-012; BV-020</x:v>
+      </x:c>
+      <x:c r="F8" s="59" t="str">
+        <x:v>docs/engineering/HEALTH-STORY-1.md</x:v>
+      </x:c>
+      <x:c r="G8" s="59" t="str">
+        <x:v>Health Story 1 local engineering complete: web/native journeys, permissions, encryption and restore verified. Clinical activation, manual accessibility, physical devices and participant signoff remain separate.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="108" customHeight="1">
+      <x:c r="A9" s="60" t="str">
+        <x:v>CJ-005</x:v>
+      </x:c>
+      <x:c r="B9" s="60" t="str">
+        <x:v>Knowledge definitions, review/activation/withdrawal ledger, privileged administration and version fixtures.</x:v>
+      </x:c>
+      <x:c r="C9" s="60" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D9" s="60" t="str">
+        <x:v>CJ-001</x:v>
+      </x:c>
+      <x:c r="E9" s="60" t="str">
+        <x:v>BV-019–BV-023; BV-034</x:v>
+      </x:c>
+      <x:c r="F9" s="60" t="str">
+        <x:v>documentation/product-experience/DELIVERY-AND-ACCEPTANCE.md</x:v>
+      </x:c>
+      <x:c r="G9" s="60" t="str">
+        <x:v>Proposed scope. No capability, clinical content activation or approval is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="108" customHeight="1">
+      <x:c r="A10" s="59" t="str">
+        <x:v>CJ-006</x:v>
+      </x:c>
+      <x:c r="B10" s="59" t="str">
+        <x:v>Focus taxonomy/mapping and evidence membership, including user collections and visible non-assessment.</x:v>
+      </x:c>
+      <x:c r="C10" s="59" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D10" s="59" t="str">
+        <x:v>CJ-003; CJ-005</x:v>
+      </x:c>
+      <x:c r="E10" s="59" t="str">
+        <x:v>BV-019–BV-023</x:v>
+      </x:c>
+      <x:c r="F10" s="59" t="str">
+        <x:v>documentation/product-experience/DELIVERY-AND-ACCEPTANCE.md</x:v>
+      </x:c>
+      <x:c r="G10" s="59" t="str">
+        <x:v>Proposed scope. No capability, clinical content activation or approval is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="108" customHeight="1">
+      <x:c r="A11" s="60" t="str">
+        <x:v>CJ-007</x:v>
+      </x:c>
+      <x:c r="B11" s="60" t="str">
+        <x:v>Connected insights, factual change detail, knowledge applicability and constrained next-step presentation.</x:v>
+      </x:c>
+      <x:c r="C11" s="60" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D11" s="60" t="str">
+        <x:v>CJ-002; CJ-005; CJ-006</x:v>
+      </x:c>
+      <x:c r="E11" s="60" t="str">
+        <x:v>BV-019–BV-023</x:v>
+      </x:c>
+      <x:c r="F11" s="60" t="str">
+        <x:v>documentation/product-experience/DELIVERY-AND-ACCEPTANCE.md</x:v>
+      </x:c>
+      <x:c r="G11" s="60" t="str">
+        <x:v>Proposed scope. No capability, clinical content activation or approval is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="108" customHeight="1">
+      <x:c r="A12" s="59" t="str">
+        <x:v>CJ-008</x:v>
+      </x:c>
+      <x:c r="B12" s="59" t="str">
+        <x:v>Contextual read tools and versioned AI citation/answer schemas for timeline, context and focus evidence.</x:v>
+      </x:c>
+      <x:c r="C12" s="59" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D12" s="59" t="str">
+        <x:v>CJ-003; CJ-007 for focus tools</x:v>
+      </x:c>
+      <x:c r="E12" s="59" t="str">
+        <x:v>BV-024–BV-028</x:v>
+      </x:c>
+      <x:c r="F12" s="59" t="str">
+        <x:v>documentation/product-experience/DELIVERY-AND-ACCEPTANCE.md</x:v>
+      </x:c>
+      <x:c r="G12" s="59" t="str">
+        <x:v>Proposed scope. No capability, clinical content activation or approval is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="108" customHeight="1">
+      <x:c r="A13" s="60" t="str">
+        <x:v>CJ-009</x:v>
+      </x:c>
+      <x:c r="B13" s="60" t="str">
+        <x:v>Wellness baseline, user goals, prospective opportunities, manual check-ins and pause/history.</x:v>
+      </x:c>
+      <x:c r="C13" s="60" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D13" s="60" t="str">
+        <x:v>CJ-001</x:v>
+      </x:c>
+      <x:c r="E13" s="60" t="str">
+        <x:v>BV-033; BV-036; BV-040</x:v>
+      </x:c>
+      <x:c r="F13" s="60" t="str">
+        <x:v>documentation/product-experience/DELIVERY-AND-ACCEPTANCE.md</x:v>
+      </x:c>
+      <x:c r="G13" s="60" t="str">
+        <x:v>Proposed scope. No capability, clinical content activation or approval is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="108" customHeight="1">
+      <x:c r="A14" s="59" t="str">
+        <x:v>CJ-010</x:v>
+      </x:c>
+      <x:c r="B14" s="59" t="str">
+        <x:v>Reviewed action catalogue and impact detail: targets, evidence, variants, restrictions and licensing.</x:v>
+      </x:c>
+      <x:c r="C14" s="59" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D14" s="59" t="str">
+        <x:v>CJ-005</x:v>
+      </x:c>
+      <x:c r="E14" s="59" t="str">
+        <x:v>BV-034</x:v>
+      </x:c>
+      <x:c r="F14" s="59" t="str">
+        <x:v>documentation/product-experience/DELIVERY-AND-ACCEPTANCE.md</x:v>
+      </x:c>
+      <x:c r="G14" s="59" t="str">
+        <x:v>Proposed scope. No capability, clinical content activation or approval is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="108" customHeight="1">
+      <x:c r="A15" s="60" t="str">
+        <x:v>CJ-011</x:v>
+      </x:c>
+      <x:c r="B15" s="60" t="str">
+        <x:v>Deterministic eligibility, consented health summary, burden-aware selection and accepted plan versioning.</x:v>
+      </x:c>
+      <x:c r="C15" s="60" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D15" s="60" t="str">
+        <x:v>CJ-002; CJ-009; CJ-010</x:v>
+      </x:c>
+      <x:c r="E15" s="60" t="str">
+        <x:v>BV-034; BV-035</x:v>
+      </x:c>
+      <x:c r="F15" s="60" t="str">
+        <x:v>documentation/product-experience/DELIVERY-AND-ACCEPTANCE.md</x:v>
+      </x:c>
+      <x:c r="G15" s="60" t="str">
+        <x:v>Proposed scope. No capability, clinical content activation or approval is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="108" customHeight="1">
+      <x:c r="A16" s="59" t="str">
+        <x:v>CJ-012</x:v>
+      </x:c>
+      <x:c r="B16" s="59" t="str">
+        <x:v>Reflection, recovery, user-confirmed adaptation and behavior/outcome view.</x:v>
+      </x:c>
+      <x:c r="C16" s="59" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D16" s="59" t="str">
+        <x:v>CJ-009; CJ-011 for recommended plans</x:v>
+      </x:c>
+      <x:c r="E16" s="59" t="str">
+        <x:v>BV-036; BV-040; BV-041</x:v>
+      </x:c>
+      <x:c r="F16" s="59" t="str">
+        <x:v>documentation/product-experience/DELIVERY-AND-ACCEPTANCE.md</x:v>
+      </x:c>
+      <x:c r="G16" s="59" t="str">
+        <x:v>Proposed scope. No capability, clinical content activation or approval is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="108" customHeight="1">
+      <x:c r="A17" s="60" t="str">
+        <x:v>CJ-013</x:v>
+      </x:c>
+      <x:c r="B17" s="60" t="str">
+        <x:v>Wellness assistant read tools and later explicit draft-to-confirmed-write proposals.</x:v>
+      </x:c>
+      <x:c r="C17" s="60" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D17" s="60" t="str">
+        <x:v>CJ-008; CJ-011; CJ-012 as applicable</x:v>
+      </x:c>
+      <x:c r="E17" s="60" t="str">
+        <x:v>BV-037</x:v>
+      </x:c>
+      <x:c r="F17" s="60" t="str">
+        <x:v>documentation/product-experience/DELIVERY-AND-ACCEPTANCE.md</x:v>
+      </x:c>
+      <x:c r="G17" s="60" t="str">
+        <x:v>Proposed scope. No capability, clinical content activation or approval is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="108" customHeight="1">
+      <x:c r="A18" s="59" t="str">
+        <x:v>CJ-014</x:v>
+      </x:c>
+      <x:c r="B18" s="59" t="str">
+        <x:v>Reviewed education and private question-saving with independent Community identity/trust boundary.</x:v>
+      </x:c>
+      <x:c r="C18" s="59" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D18" s="59" t="str">
+        <x:v>CJ-005; CJ-002 for private question records</x:v>
+      </x:c>
+      <x:c r="E18" s="59" t="str">
+        <x:v>BV-042; BV-043; BV-045</x:v>
+      </x:c>
+      <x:c r="F18" s="59" t="str">
+        <x:v>documentation/product-experience/DELIVERY-AND-ACCEPTANCE.md</x:v>
+      </x:c>
+      <x:c r="G18" s="59" t="str">
+        <x:v>Proposed scope. No capability, clinical content activation or approval is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="108" customHeight="1">
+      <x:c r="A19" s="60" t="str">
+        <x:v>CJ-015</x:v>
+      </x:c>
+      <x:c r="B19" s="60" t="str">
+        <x:v>Cross-module generation/invalidation, data lifecycle, privacy-aware search, restore/rebuild and operational metrics.</x:v>
+      </x:c>
+      <x:c r="C19" s="60" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="D19" s="60" t="str">
+        <x:v>CJ-001 onward, incrementally</x:v>
+      </x:c>
+      <x:c r="E19" s="60" t="str">
+        <x:v>BV-011; BV-029–BV-031; BV-047–BV-048</x:v>
+      </x:c>
+      <x:c r="F19" s="60" t="str">
+        <x:v>docs/engineering/HEALTH-STORY-1.md</x:v>
+      </x:c>
+      <x:c r="G19" s="60" t="str">
+        <x:v>J1 includes source invalidation, permissions and encrypted restore. Future module invalidation and wider lifecycle work remain.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="108" customHeight="1">
+      <x:c r="A20" s="59" t="str">
+        <x:v>CJ-016</x:v>
+      </x:c>
+      <x:c r="B20" s="59" t="str">
+        <x:v>Web/native journey QA, accessibility, comprehension study plan, content/claims review and staged rollout evidence.</x:v>
+      </x:c>
+      <x:c r="C20" s="59" t="str">
+        <x:v>In Progress</x:v>
+      </x:c>
+      <x:c r="D20" s="59" t="str">
+        <x:v>Each slice; final integrated run</x:v>
+      </x:c>
+      <x:c r="E20" s="59" t="str">
+        <x:v>BV-029–BV-032; BV-041; BV-049–BV-051</x:v>
+      </x:c>
+      <x:c r="F20" s="59" t="str">
+        <x:v>docs/engineering/HEALTH-STORY-1.md</x:v>
+      </x:c>
+      <x:c r="G20" s="59" t="str">
+        <x:v>J1 automated QA recorded; manual accessibility, physical devices, participants and final integrated rollout remain.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="108" customHeight="1">
+      <x:c r="A21" s="60" t="str">
+        <x:v>CJ-017</x:v>
+      </x:c>
+      <x:c r="B21" s="60" t="str">
+        <x:v>Optional manual-vital expansion, device connectors and preference-driven delivered reminders.</x:v>
+      </x:c>
+      <x:c r="C21" s="60" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D21" s="60" t="str">
+        <x:v>CJ-003; CJ-009; separate consent/operations design</x:v>
+      </x:c>
+      <x:c r="E21" s="60" t="str">
+        <x:v>BV-038; BV-039</x:v>
+      </x:c>
+      <x:c r="F21" s="60" t="str">
+        <x:v>documentation/product-experience/DELIVERY-AND-ACCEPTANCE.md</x:v>
+      </x:c>
+      <x:c r="G21" s="60" t="str">
+        <x:v>Proposed scope. No capability, clinical content activation or approval is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="108" customHeight="1">
+      <x:c r="A22" s="59" t="str">
+        <x:v>CJ-018</x:v>
+      </x:c>
+      <x:c r="B22" s="59" t="str">
+        <x:v>Optional professional submissions and moderated community participation.</x:v>
+      </x:c>
+      <x:c r="C22" s="59" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="D22" s="59" t="str">
+        <x:v>CJ-014; staffed moderation and policy</x:v>
+      </x:c>
+      <x:c r="E22" s="59" t="str">
+        <x:v>BV-044–BV-046</x:v>
+      </x:c>
+      <x:c r="F22" s="59" t="str">
+        <x:v>documentation/product-experience/DELIVERY-AND-ACCEPTANCE.md</x:v>
+      </x:c>
+      <x:c r="G22" s="59" t="str">
+        <x:v>Proposed scope. No capability, clinical content activation or approval is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="52"/>
+      <x:c r="B23" s="52"/>
+      <x:c r="C23" s="52"/>
+      <x:c r="D23" s="52"/>
+      <x:c r="E23" s="52"/>
+      <x:c r="F23" s="52"/>
+      <x:c r="G23" s="52"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="62" t="str">
+        <x:v>Source: Connected journey delivery plan; Health Story 1 implementation evidence.</x:v>
+      </x:c>
+      <x:c r="B24" s="52"/>
+      <x:c r="C24" s="52"/>
+      <x:c r="D24" s="52"/>
+      <x:c r="E24" s="52"/>
+      <x:c r="F24" s="52"/>
+      <x:c r="G24" s="52"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="62" t="str">
+        <x:v>Human research, clinical/content activation and platform acceptance remain separate gates.</x:v>
+      </x:c>
+      <x:c r="B25" s="52"/>
+      <x:c r="C25" s="52"/>
+      <x:c r="D25" s="52"/>
+      <x:c r="E25" s="52"/>
+      <x:c r="F25" s="52"/>
+      <x:c r="G25" s="52"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="C5:C22">
+      <x:formula1>"Backlog,Ready,In Progress,In Review,Done,Blocked"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>